<commit_message>
fix non reguler cutah & hometrip & update git ignore
</commit_message>
<xml_diff>
--- a/e2e/data/test-data-nonregular.xlsx
+++ b/e2e/data/test-data-nonregular.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Work\Telkomcel\test\e2e\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{76D89F6E-CD1C-4234-B786-61443FEADCE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54A69629-C516-4137-A5B8-DBD4FB0DF72E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="12210" windowHeight="12885" firstSheet="5" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="705" yWindow="5505" windowWidth="23775" windowHeight="10140" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Bfkj" sheetId="1" r:id="rId1"/>
@@ -188,30 +188,12 @@
     <t>0.5</t>
   </si>
   <si>
-    <t>170</t>
-  </si>
-  <si>
     <t>0.25</t>
   </si>
   <si>
-    <t>45</t>
-  </si>
-  <si>
     <t>150</t>
   </si>
   <si>
-    <t>350</t>
-  </si>
-  <si>
-    <t>280</t>
-  </si>
-  <si>
-    <t>105</t>
-  </si>
-  <si>
-    <t>252</t>
-  </si>
-  <si>
     <t>1</t>
   </si>
   <si>
@@ -263,24 +245,12 @@
     <t>2026-06</t>
   </si>
   <si>
-    <t>14.17</t>
-  </si>
-  <si>
     <t>0.75</t>
   </si>
   <si>
-    <t>21.25</t>
-  </si>
-  <si>
-    <t>28.33</t>
-  </si>
-  <si>
     <t>2026-07</t>
   </si>
   <si>
-    <t>58.33</t>
-  </si>
-  <si>
     <t>january</t>
   </si>
   <si>
@@ -288,6 +258,36 @@
   </si>
   <si>
     <t>maret</t>
+  </si>
+  <si>
+    <t>20.83</t>
+  </si>
+  <si>
+    <t>52.08</t>
+  </si>
+  <si>
+    <t>93.75</t>
+  </si>
+  <si>
+    <t>135.42</t>
+  </si>
+  <si>
+    <t>177.09</t>
+  </si>
+  <si>
+    <t>218.76</t>
+  </si>
+  <si>
+    <t>260.43</t>
+  </si>
+  <si>
+    <t>125.00</t>
+  </si>
+  <si>
+    <t>250.00</t>
+  </si>
+  <si>
+    <t>500.00</t>
   </si>
 </sst>
 </file>
@@ -1170,6 +1170,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:F24"/>
   <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="3" max="3" width="35.5" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
@@ -1812,7 +1815,7 @@
         <v>49</v>
       </c>
       <c r="I5" s="1" t="s">
-        <v>50</v>
+        <v>82</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
@@ -1838,10 +1841,10 @@
         <v>41</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="I6" s="1" t="s">
-        <v>52</v>
+        <v>81</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
@@ -1870,7 +1873,7 @@
         <v>49</v>
       </c>
       <c r="I7" s="1" t="s">
-        <v>53</v>
+        <v>82</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
@@ -1899,7 +1902,7 @@
         <v>49</v>
       </c>
       <c r="I8" s="1" t="s">
-        <v>54</v>
+        <v>82</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
@@ -1928,7 +1931,7 @@
         <v>49</v>
       </c>
       <c r="I9" s="1" t="s">
-        <v>54</v>
+        <v>82</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
@@ -1957,7 +1960,7 @@
         <v>49</v>
       </c>
       <c r="I10" s="1" t="s">
-        <v>53</v>
+        <v>82</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
@@ -1986,7 +1989,7 @@
         <v>49</v>
       </c>
       <c r="I11" s="1" t="s">
-        <v>55</v>
+        <v>82</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
@@ -2012,10 +2015,10 @@
         <v>45</v>
       </c>
       <c r="H12" s="1" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="I12" s="1" t="s">
-        <v>45</v>
+        <v>83</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
@@ -2044,7 +2047,7 @@
         <v>49</v>
       </c>
       <c r="I13" s="1" t="s">
-        <v>56</v>
+        <v>82</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
@@ -2073,7 +2076,7 @@
         <v>49</v>
       </c>
       <c r="I14" s="1" t="s">
-        <v>57</v>
+        <v>82</v>
       </c>
     </row>
   </sheetData>
@@ -2233,22 +2236,22 @@
         <v>23</v>
       </c>
       <c r="E5" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="F5" t="s">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="G5" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
       <c r="H5" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
       <c r="I5" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
       <c r="J5" t="s">
-        <v>62</v>
+        <v>56</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
@@ -2268,16 +2271,16 @@
         <v>42</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
       <c r="I6" s="1" t="s">
-        <v>64</v>
+        <v>58</v>
       </c>
       <c r="J6" s="1" t="s">
         <v>40</v>
@@ -2297,19 +2300,19 @@
         <v>23</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>65</v>
+        <v>59</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>64</v>
+        <v>58</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
       <c r="I7" s="1" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="J7" s="1" t="s">
         <v>41</v>
@@ -2329,19 +2332,19 @@
         <v>23</v>
       </c>
       <c r="E8" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="F8" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="F8" s="1" t="s">
-        <v>66</v>
-      </c>
       <c r="G8" s="1" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="H8" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
       <c r="I8" s="1" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
       <c r="J8" s="1" t="s">
         <v>42</v>
@@ -2361,19 +2364,19 @@
         <v>23</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>67</v>
+        <v>61</v>
       </c>
       <c r="F9" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="H9" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
       <c r="I9" s="1" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
       <c r="J9" s="1" t="s">
         <v>43</v>
@@ -2393,19 +2396,19 @@
         <v>23</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>67</v>
+        <v>61</v>
       </c>
       <c r="F10" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
       <c r="H10" s="1" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="I10" s="1" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
       <c r="J10" s="1" t="s">
         <v>43</v>
@@ -2425,19 +2428,19 @@
         <v>23</v>
       </c>
       <c r="E11" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="F11" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="F11" s="1" t="s">
-        <v>66</v>
-      </c>
       <c r="G11" s="1" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
       <c r="H11" s="1" t="s">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="I11" s="1" t="s">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="J11" s="1" t="s">
         <v>42</v>
@@ -2457,22 +2460,22 @@
         <v>23</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>64</v>
+        <v>58</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
       <c r="H12" s="1" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
       <c r="I12" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="J12" s="1" t="s">
         <v>66</v>
-      </c>
-      <c r="J12" s="1" t="s">
-        <v>72</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.25">
@@ -2492,16 +2495,16 @@
         <v>45</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>64</v>
+        <v>58</v>
       </c>
       <c r="G13" s="1" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
       <c r="H13" s="1" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
       <c r="I13" s="1" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
       <c r="J13" s="1" t="s">
         <v>45</v>
@@ -2521,19 +2524,19 @@
         <v>23</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="G14" s="1" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
       <c r="H14" s="1" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
       <c r="I14" s="1" t="s">
-        <v>64</v>
+        <v>58</v>
       </c>
       <c r="J14" s="1" t="s">
         <v>46</v>
@@ -2553,22 +2556,22 @@
         <v>23</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>69</v>
+        <v>63</v>
       </c>
       <c r="F15" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="G15" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="H15" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="I15" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="J15" s="1" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
     </row>
   </sheetData>
@@ -2686,7 +2689,7 @@
         <v>49</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
@@ -2703,10 +2706,10 @@
         <v>24</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>76</v>
+        <v>69</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
@@ -2723,10 +2726,10 @@
         <v>25</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
@@ -2740,13 +2743,13 @@
         <v>22</v>
       </c>
       <c r="D8" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
@@ -2763,7 +2766,7 @@
         <v>31</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="F9" s="1" t="s">
         <v>78</v>
@@ -2780,13 +2783,13 @@
         <v>22</v>
       </c>
       <c r="D10" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
@@ -2800,10 +2803,10 @@
         <v>37</v>
       </c>
       <c r="D11" t="s">
-        <v>79</v>
+        <v>70</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="F11" s="1" t="s">
         <v>80</v>
@@ -2951,7 +2954,7 @@
         <v>200</v>
       </c>
       <c r="G5" t="s">
-        <v>81</v>
+        <v>71</v>
       </c>
       <c r="H5">
         <v>400</v>
@@ -2977,7 +2980,7 @@
         <v>250</v>
       </c>
       <c r="G6" t="s">
-        <v>82</v>
+        <v>72</v>
       </c>
       <c r="H6">
         <v>500</v>
@@ -3003,7 +3006,7 @@
         <v>250</v>
       </c>
       <c r="G7" t="s">
-        <v>83</v>
+        <v>73</v>
       </c>
       <c r="H7">
         <v>500</v>

</xml_diff>

<commit_message>
fix non reguler - tunjangan kompetensi
</commit_message>
<xml_diff>
--- a/e2e/data/test-data-nonregular.xlsx
+++ b/e2e/data/test-data-nonregular.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Work\Telkomcel\test\e2e\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54A69629-C516-4137-A5B8-DBD4FB0DF72E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{530C4511-056D-4F84-9A2F-D6861ED93E49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="705" yWindow="5505" windowWidth="23775" windowHeight="10140" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="225" yWindow="2340" windowWidth="23775" windowHeight="10140" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Bfkj" sheetId="1" r:id="rId1"/>
@@ -272,15 +272,6 @@
     <t>135.42</t>
   </si>
   <si>
-    <t>177.09</t>
-  </si>
-  <si>
-    <t>218.76</t>
-  </si>
-  <si>
-    <t>260.43</t>
-  </si>
-  <si>
     <t>125.00</t>
   </si>
   <si>
@@ -288,6 +279,15 @@
   </si>
   <si>
     <t>500.00</t>
+  </si>
+  <si>
+    <t>218.75</t>
+  </si>
+  <si>
+    <t>177.08</t>
+  </si>
+  <si>
+    <t>41.67</t>
   </si>
 </sst>
 </file>
@@ -1815,7 +1815,7 @@
         <v>49</v>
       </c>
       <c r="I5" s="1" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
@@ -1844,7 +1844,7 @@
         <v>50</v>
       </c>
       <c r="I6" s="1" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
@@ -1873,7 +1873,7 @@
         <v>49</v>
       </c>
       <c r="I7" s="1" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
@@ -1902,7 +1902,7 @@
         <v>49</v>
       </c>
       <c r="I8" s="1" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
@@ -1931,7 +1931,7 @@
         <v>49</v>
       </c>
       <c r="I9" s="1" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
@@ -1960,7 +1960,7 @@
         <v>49</v>
       </c>
       <c r="I10" s="1" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
@@ -1989,7 +1989,7 @@
         <v>49</v>
       </c>
       <c r="I11" s="1" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
@@ -2018,7 +2018,7 @@
         <v>52</v>
       </c>
       <c r="I12" s="1" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
@@ -2047,7 +2047,7 @@
         <v>49</v>
       </c>
       <c r="I13" s="1" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
@@ -2076,7 +2076,7 @@
         <v>49</v>
       </c>
       <c r="I14" s="1" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
     </row>
   </sheetData>
@@ -2769,7 +2769,7 @@
         <v>52</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
@@ -2789,7 +2789,7 @@
         <v>52</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
@@ -2809,7 +2809,7 @@
         <v>52</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix bug and add test compare report
</commit_message>
<xml_diff>
--- a/e2e/data/test-data-nonregular.xlsx
+++ b/e2e/data/test-data-nonregular.xlsx
@@ -2683,7 +2683,7 @@
         <v>february</v>
       </c>
       <c r="H6">
-        <v>500</v>
+        <v>650</v>
       </c>
     </row>
     <row r="7">
@@ -2709,11 +2709,10 @@
         <v>maret</v>
       </c>
       <c r="H7">
-        <v>500</v>
+        <v>900</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:H7"/>
   </ignoredErrors>

</xml_diff>